<commit_message>
total 89 papers downloaded
</commit_message>
<xml_diff>
--- a/Classification/Classification.xlsx
+++ b/Classification/Classification.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Jihad\Skin-cancer-papers\Classification\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3D63EEC-2CA4-4EEB-8079-01454D031D41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F7988FA-5264-4C3E-80C9-19447AE05AA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2268" yWindow="2268" windowWidth="17280" windowHeight="8964" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="6276" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="93">
   <si>
     <t>Serial</t>
   </si>
@@ -156,6 +156,156 @@
   </si>
   <si>
     <t>transfer learning</t>
+  </si>
+  <si>
+    <t>Melanoma diagnosis using deep learning techniques on dermatoscopic images</t>
+  </si>
+  <si>
+    <t>https://link.springer.com/article/10.1186/s12880-020-00534-8</t>
+  </si>
+  <si>
+    <t>Cancer-Net SCa tailored deep neural network designs for detection of skin cancer from dermoscopy image</t>
+  </si>
+  <si>
+    <t>https://link.springer.com/article/10.1186/s12880-022-00871-w?utm_source=chatgpt.com</t>
+  </si>
+  <si>
+    <t>Detection of Skin Cancer Based on Skin Lesion Images Using Deep Learning</t>
+  </si>
+  <si>
+    <t>https://www.mdpi.com/2227-9032/10/7/1183</t>
+  </si>
+  <si>
+    <t>SCDNet: A Deep Learning-Based Framework for the Multiclassification of Skin Cancer Using Dermoscopy Images</t>
+  </si>
+  <si>
+    <t>https://www.mdpi.com/1424-8220/22/15/5652</t>
+  </si>
+  <si>
+    <t>Multiclass Skin Lesion Classification Using a Novel Lightweight Deep Learning Framework for Smart Healthcare</t>
+  </si>
+  <si>
+    <t>https://www.mdpi.com/2076-3417/12/5/2677</t>
+  </si>
+  <si>
+    <t>Machine Learning and Deep Learning Algorithms for Skin Cancer Classification from Dermoscopic Images</t>
+  </si>
+  <si>
+    <t>https://www.mdpi.com/2306-5354/9/3/97</t>
+  </si>
+  <si>
+    <t>Skin lesion classification of dermoscopic images using machine learning and convolutional neural network</t>
+  </si>
+  <si>
+    <t>https://www.nature.com/articles/s41598-022-22644-9</t>
+  </si>
+  <si>
+    <t>https://www.mdpi.com/1424-8220/22/11/4008</t>
+  </si>
+  <si>
+    <t>An Effective Skin Cancer Classification Mechanism via Medical Vision Transformer</t>
+  </si>
+  <si>
+    <t>https://www.mdpi.com/1424-8220/22/19/7530</t>
+  </si>
+  <si>
+    <t>Skin Lesion Classification on Imbalanced Data Using Deep Learning with Soft Attention</t>
+  </si>
+  <si>
+    <t>Skin Lesion Classification Using Collective Intelligence of Multiple Neural Networks</t>
+  </si>
+  <si>
+    <t>https://www.mdpi.com/1424-8220/22/12/4399</t>
+  </si>
+  <si>
+    <t>Multiclass Skin Lesion Classification Using Hybrid Deep Features Selection and Extreme Learning Machine</t>
+  </si>
+  <si>
+    <t>https://www.mdpi.com/1424-8220/22/3/799</t>
+  </si>
+  <si>
+    <t>Melanoma Classification Using a Novel Deep Convolutional Neural Network with Dermoscopy Images</t>
+  </si>
+  <si>
+    <t>https://www.mdpi.com/1424-8220/22/3/1134</t>
+  </si>
+  <si>
+    <t>Dermoscopic Image Classification Method Using an Ensemble of Fine-Tuned Convolutional Neural Networks</t>
+  </si>
+  <si>
+    <t>https://www.mdpi.com/1424-8220/22/11/4147</t>
+  </si>
+  <si>
+    <t>A novel framework of multiclass skin lesion recognition from dermoscopic images using deep learning and explainable AI</t>
+  </si>
+  <si>
+    <t>https://www.frontiersin.org/journals/oncology/articles/10.3389/fonc.2023.1151257/full</t>
+  </si>
+  <si>
+    <t>Detection for melanoma skin cancer through ACCF, BPPF, and CLF techniques with machine learning approach</t>
+  </si>
+  <si>
+    <t>https://link.springer.com/article/10.1186/s12859-023-05584-7</t>
+  </si>
+  <si>
+    <t>Radiomic and deep learning analysis of dermoscopic images for skin lesion pattern decoding</t>
+  </si>
+  <si>
+    <t>https://www.nature.com/articles/s41598-024-70231-x?utm_source=chatgpt.com</t>
+  </si>
+  <si>
+    <t>Hybrid Deep Learning Framework for Melanoma Diagnosis and Classification</t>
+  </si>
+  <si>
+    <t>https://www.mdpi.com/2075-4418/14/19/2242</t>
+  </si>
+  <si>
+    <t>SkinSwinViT: A Lightweight Transformer-Based Method for Multiclass Skin Lesion Classification with Enhanced Generalization Capabilities</t>
+  </si>
+  <si>
+    <t>https://www.mdpi.com/2076-3417/14/10/4005</t>
+  </si>
+  <si>
+    <t>Towards unbiased skin cancer classification using deep feature fusion</t>
+  </si>
+  <si>
+    <t>https://link.springer.com/article/10.1186/s12911-025-02889-w?utm_source=chatgpt.com</t>
+  </si>
+  <si>
+    <t>Multiclass skin lesion classification and localziation from dermoscopic images using a novel network-level fused deep architecture and explainable artificial intelligence</t>
+  </si>
+  <si>
+    <t>https://link.springer.com/article/10.1186/s12911-025-03051-2?utm_source=chatgpt.com</t>
+  </si>
+  <si>
+    <t>A deep learning framework for automated early diagnosis and classification of skin cancer lesions in dermoscopy images</t>
+  </si>
+  <si>
+    <t>https://www.nature.com/articles/s41598-025-15655-9?utm_source=chatgpt.com</t>
+  </si>
+  <si>
+    <t>Explainable deep learning approaches for high precision early melanoma detection using dermoscopic images</t>
+  </si>
+  <si>
+    <t>https://www.nature.com/articles/s41598-025-09938-4?utm_source=chatgpt.com</t>
+  </si>
+  <si>
+    <t>Federated learning for privacy-preserving skin cancer classification using deep neural networks</t>
+  </si>
+  <si>
+    <t>https://www.frontiersin.org/journals/oncology/articles/10.3389/fonc.2026.1720748/full</t>
+  </si>
+  <si>
+    <t>Advancing skin cancer detection through deep learning and fusion of patient metadata and skin lesion images</t>
+  </si>
+  <si>
+    <t>https://www.nature.com/articles/s41598-025-26392-4?utm_source=chatgpt.com</t>
+  </si>
+  <si>
+    <t>DermaScanAI an explainable hybrid deep learning framework for automated skin lesion classification using dual attention and metadata fusion</t>
+  </si>
+  <si>
+    <t>https://www.nature.com/articles/s41598-026-46011-0?utm_source=chatgpt.com</t>
   </si>
 </sst>
 </file>
@@ -206,7 +356,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -216,6 +366,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -498,7 +651,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="E5:I31"/>
+  <dimension ref="E5:I66"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="4" width="8.88671875" style="1"/>
@@ -753,7 +906,7 @@
         <v>14</v>
       </c>
       <c r="F19" s="1">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="G19" s="1" t="s">
         <v>38</v>
@@ -769,6 +922,9 @@
       <c r="E20" s="1">
         <v>15</v>
       </c>
+      <c r="F20" s="1">
+        <v>2024</v>
+      </c>
       <c r="G20" s="1" t="s">
         <v>40</v>
       </c>
@@ -779,59 +935,531 @@
         <v>41</v>
       </c>
     </row>
-    <row r="21" spans="5:9" x14ac:dyDescent="0.3">
+    <row r="21" spans="5:9" ht="100.8" x14ac:dyDescent="0.3">
       <c r="E21" s="1">
         <v>16</v>
       </c>
-    </row>
-    <row r="22" spans="5:9" x14ac:dyDescent="0.3">
+      <c r="F21" s="1">
+        <v>2021</v>
+      </c>
+      <c r="G21" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="H21" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I21" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="22" spans="5:9" ht="144" x14ac:dyDescent="0.3">
       <c r="E22" s="1">
         <v>17</v>
       </c>
-    </row>
-    <row r="23" spans="5:9" x14ac:dyDescent="0.3">
+      <c r="F22" s="1">
+        <v>2022</v>
+      </c>
+      <c r="G22" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="H22" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I22" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="23" spans="5:9" ht="86.4" x14ac:dyDescent="0.3">
       <c r="E23" s="1">
         <v>18</v>
       </c>
-    </row>
-    <row r="24" spans="5:9" x14ac:dyDescent="0.3">
+      <c r="G23" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="H23" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I23" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="24" spans="5:9" ht="144" x14ac:dyDescent="0.3">
       <c r="E24" s="1">
         <v>19</v>
       </c>
-    </row>
-    <row r="25" spans="5:9" x14ac:dyDescent="0.3">
+      <c r="F24" s="1">
+        <v>2022</v>
+      </c>
+      <c r="G24" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="H24" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I24" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="25" spans="5:9" ht="129.6" x14ac:dyDescent="0.3">
       <c r="E25" s="1">
         <v>20</v>
       </c>
-    </row>
-    <row r="26" spans="5:9" x14ac:dyDescent="0.3">
+      <c r="F25" s="1">
+        <v>2022</v>
+      </c>
+      <c r="G25" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="H25" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I25" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="26" spans="5:9" ht="129.6" x14ac:dyDescent="0.3">
       <c r="E26" s="1">
         <v>21</v>
       </c>
-    </row>
-    <row r="27" spans="5:9" x14ac:dyDescent="0.3">
+      <c r="F26" s="1">
+        <v>2022</v>
+      </c>
+      <c r="G26" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="H26" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="I26" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="27" spans="5:9" ht="144" x14ac:dyDescent="0.3">
       <c r="E27" s="1">
         <v>22</v>
       </c>
-    </row>
-    <row r="28" spans="5:9" x14ac:dyDescent="0.3">
+      <c r="F27" s="1">
+        <v>2022</v>
+      </c>
+      <c r="G27" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="H27" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="I27" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="28" spans="5:9" ht="100.8" x14ac:dyDescent="0.3">
       <c r="E28" s="1">
         <v>23</v>
       </c>
-    </row>
-    <row r="29" spans="5:9" x14ac:dyDescent="0.3">
+      <c r="F28" s="1">
+        <v>2022</v>
+      </c>
+      <c r="G28" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="H28" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I28" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="29" spans="5:9" ht="115.2" x14ac:dyDescent="0.3">
       <c r="E29" s="1">
         <v>24</v>
       </c>
-    </row>
-    <row r="30" spans="5:9" x14ac:dyDescent="0.3">
+      <c r="F29" s="1">
+        <v>2022</v>
+      </c>
+      <c r="G29" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="H29" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I29" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="30" spans="5:9" ht="115.2" x14ac:dyDescent="0.3">
       <c r="E30" s="1">
         <v>25</v>
       </c>
-    </row>
-    <row r="31" spans="5:9" x14ac:dyDescent="0.3">
+      <c r="F30" s="1">
+        <v>2022</v>
+      </c>
+      <c r="G30" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="H30" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I30" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="31" spans="5:9" ht="144" x14ac:dyDescent="0.3">
       <c r="E31" s="1">
         <v>26</v>
+      </c>
+      <c r="F31" s="1">
+        <v>2022</v>
+      </c>
+      <c r="G31" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="H31" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I31" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="32" spans="5:9" ht="129.6" x14ac:dyDescent="0.3">
+      <c r="E32" s="1">
+        <v>27</v>
+      </c>
+      <c r="F32" s="1">
+        <v>2022</v>
+      </c>
+      <c r="G32" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="H32" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I32" s="1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="33" spans="5:9" ht="129.6" x14ac:dyDescent="0.3">
+      <c r="E33" s="1">
+        <v>28</v>
+      </c>
+      <c r="F33" s="1">
+        <v>2022</v>
+      </c>
+      <c r="G33" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="H33" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I33" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="34" spans="5:9" ht="158.4" x14ac:dyDescent="0.3">
+      <c r="E34" s="1">
+        <v>29</v>
+      </c>
+      <c r="F34" s="1">
+        <v>2023</v>
+      </c>
+      <c r="G34" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="H34" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I34" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="35" spans="5:9" ht="129.6" x14ac:dyDescent="0.3">
+      <c r="E35" s="1">
+        <v>30</v>
+      </c>
+      <c r="F35" s="1">
+        <v>2023</v>
+      </c>
+      <c r="G35" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="H35" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="I35" s="1" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="36" spans="5:9" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="E36" s="1">
+        <v>31</v>
+      </c>
+      <c r="F36" s="1">
+        <v>2024</v>
+      </c>
+      <c r="G36" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="H36" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I36" s="1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="37" spans="5:9" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="E37" s="1">
+        <v>32</v>
+      </c>
+      <c r="F37" s="1">
+        <v>2024</v>
+      </c>
+      <c r="G37" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="H37" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I37" s="3" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="38" spans="5:9" ht="172.8" x14ac:dyDescent="0.3">
+      <c r="E38" s="1">
+        <v>33</v>
+      </c>
+      <c r="F38" s="1">
+        <v>2024</v>
+      </c>
+      <c r="G38" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="H38" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I38" s="1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="39" spans="5:9" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="E39" s="1">
+        <v>34</v>
+      </c>
+      <c r="F39" s="1">
+        <v>2025</v>
+      </c>
+      <c r="G39" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="H39" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I39" s="1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="40" spans="5:9" ht="230.4" x14ac:dyDescent="0.3">
+      <c r="E40" s="1">
+        <v>35</v>
+      </c>
+      <c r="F40" s="1">
+        <v>2025</v>
+      </c>
+      <c r="G40" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="H40" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I40" s="1" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="41" spans="5:9" ht="172.8" x14ac:dyDescent="0.3">
+      <c r="E41" s="1">
+        <v>36</v>
+      </c>
+      <c r="F41" s="1">
+        <v>2025</v>
+      </c>
+      <c r="G41" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="H41" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I41" s="1" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="42" spans="5:9" ht="158.4" x14ac:dyDescent="0.3">
+      <c r="E42" s="1">
+        <v>37</v>
+      </c>
+      <c r="F42" s="1">
+        <v>2025</v>
+      </c>
+      <c r="G42" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="H42" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I42" s="1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="43" spans="5:9" ht="129.6" x14ac:dyDescent="0.3">
+      <c r="E43" s="1">
+        <v>38</v>
+      </c>
+      <c r="F43" s="1">
+        <v>2026</v>
+      </c>
+      <c r="G43" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="H43" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I43" s="1" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="44" spans="5:9" ht="144" x14ac:dyDescent="0.3">
+      <c r="E44" s="1">
+        <v>39</v>
+      </c>
+      <c r="F44" s="1">
+        <v>2026</v>
+      </c>
+      <c r="G44" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="H44" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I44" s="1" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="45" spans="5:9" ht="201.6" x14ac:dyDescent="0.3">
+      <c r="E45" s="1">
+        <v>40</v>
+      </c>
+      <c r="F45" s="1">
+        <v>2026</v>
+      </c>
+      <c r="G45" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="H45" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I45" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="46" spans="5:9" x14ac:dyDescent="0.3">
+      <c r="E46" s="1">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="47" spans="5:9" x14ac:dyDescent="0.3">
+      <c r="E47" s="1">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="48" spans="5:9" x14ac:dyDescent="0.3">
+      <c r="E48" s="1">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="49" spans="5:5" x14ac:dyDescent="0.3">
+      <c r="E49" s="1">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="50" spans="5:5" x14ac:dyDescent="0.3">
+      <c r="E50" s="1">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="51" spans="5:5" x14ac:dyDescent="0.3">
+      <c r="E51" s="1">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="52" spans="5:5" x14ac:dyDescent="0.3">
+      <c r="E52" s="1">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="53" spans="5:5" x14ac:dyDescent="0.3">
+      <c r="E53" s="1">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="54" spans="5:5" x14ac:dyDescent="0.3">
+      <c r="E54" s="1">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="55" spans="5:5" x14ac:dyDescent="0.3">
+      <c r="E55" s="1">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="56" spans="5:5" x14ac:dyDescent="0.3">
+      <c r="E56" s="1">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="57" spans="5:5" x14ac:dyDescent="0.3">
+      <c r="E57" s="1">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="58" spans="5:5" x14ac:dyDescent="0.3">
+      <c r="E58" s="1">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="59" spans="5:5" x14ac:dyDescent="0.3">
+      <c r="E59" s="1">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="60" spans="5:5" x14ac:dyDescent="0.3">
+      <c r="E60" s="1">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="61" spans="5:5" x14ac:dyDescent="0.3">
+      <c r="E61" s="1">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="62" spans="5:5" x14ac:dyDescent="0.3">
+      <c r="E62" s="1">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="63" spans="5:5" x14ac:dyDescent="0.3">
+      <c r="E63" s="1">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="64" spans="5:5" x14ac:dyDescent="0.3">
+      <c r="E64" s="1">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="65" spans="5:5" x14ac:dyDescent="0.3">
+      <c r="E65" s="1">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="66" spans="5:5" x14ac:dyDescent="0.3">
+      <c r="E66" s="1">
+        <v>61</v>
       </c>
     </row>
   </sheetData>
@@ -839,8 +1467,10 @@
     <hyperlink ref="I11" r:id="rId1" xr:uid="{AA35B801-4513-4EEB-AE9D-AABE85B3569A}"/>
     <hyperlink ref="I18" r:id="rId2" xr:uid="{3B85DE05-8D83-4BB4-AEEB-EA43EB3EFC55}"/>
     <hyperlink ref="I20" r:id="rId3" xr:uid="{4B33EB10-E74D-49DB-BF39-F58E6176BB00}"/>
+    <hyperlink ref="I27" r:id="rId4" xr:uid="{CD489681-010B-4FEC-A585-25162A9F8D28}"/>
+    <hyperlink ref="I37" r:id="rId5" xr:uid="{79434221-9916-4D13-A4AD-DCC3DDF8472E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId4"/>
+  <pageSetup orientation="portrait" r:id="rId6"/>
 </worksheet>
 </file>
</xml_diff>